<commit_message>
fix: repair only defaulted chart axes
Axes are fixed by role so scatter charts work, and right/top or secondary
axes are left untouched. Goldens regenerated for the corrected chart axes.
</commit_message>
<xml_diff>
--- a/tests/assets/golden/win32com/test_template_1_filled.xlsx
+++ b/tests/assets/golden/win32com/test_template_1_filled.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\botti\Desktop\fillxl\tests\assets\golden\win32com\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{536D528E-9360-4F28-A159-21F76458D34E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E398E34F-438D-4CC8-A03A-C581515E0331}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -204,9 +204,6 @@
   </cellStyles>
   <dxfs count="4">
     <dxf>
-      <numFmt numFmtId="13" formatCode="0%"/>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill>
           <bgColor rgb="FFFF0000"/>
@@ -225,6 +222,9 @@
       </fill>
     </dxf>
     <dxf>
+      <numFmt numFmtId="13" formatCode="0%"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
   </dxfs>
@@ -250,7 +250,7 @@
     <tableColumn id="4" xr3:uid="{A27FC0AD-C78D-4FD1-8F51-927E6F09246C}" name="ColFormula" dataDxfId="3">
       <calculatedColumnFormula>TableTest[[#This Row],[Col1]]+TableTest[[#This Row],[Col2]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{5F1BCF14-F6A1-49D7-BDC5-54D278E411A4}" name="TestFormattedPct" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{5F1BCF14-F6A1-49D7-BDC5-54D278E411A4}" name="TestFormattedPct" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -690,13 +690,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:E6">
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="between">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="between">
       <formula>7</formula>
       <formula>7</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B6">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="between">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="between">
       <formula>2</formula>
       <formula>3</formula>
     </cfRule>

</xml_diff>